<commit_message>
modify a data standard file
</commit_message>
<xml_diff>
--- a/dama/cases/营收系统数据标准/ODS层/2 服务类/2.5 统计分析数据/报表信息/2. 应收明细报表.xlsx
+++ b/dama/cases/营收系统数据标准/ODS层/2 服务类/2.5 统计分析数据/报表信息/2. 应收明细报表.xlsx
@@ -565,7 +565,7 @@
     <t>ACC_MONEY</t>
   </si>
   <si>
-    <t>该统计分类维度下产生的应收总金额（单位：元）。</t>
+    <t>该统计分类维度下产生的应收总金额，即pi1_money+pi2_money+pi3_money+pi4_money+pi5_money+pi6_money+pi9_money（单位：元）。</t>
   </si>
   <si>
     <t>允许为空；保留2位小数。</t>
@@ -691,7 +691,7 @@
     <t>PI9_MONEY</t>
   </si>
   <si>
-    <t>特种或特殊政策自定义附加阶梯产生的费用金额（预留扩展）。</t>
+    <t>呆账。</t>
   </si>
 </sst>
 </file>
@@ -704,7 +704,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -745,13 +745,6 @@
       <color rgb="FF000000"/>
       <name val="Microsoft YaHei"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1321,48 +1314,51 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="18" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="22" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
@@ -1372,97 +1368,94 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>

</xml_diff>